<commit_message>
Redesign workbook presentation for order summary output
</commit_message>
<xml_diff>
--- a/sku_master.xlsx
+++ b/sku_master.xlsx
@@ -5,17 +5,30 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\coyot\Documents\Codex\2026-05-15\in-codex-start-a-new-repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CA9B2BC-B9F5-453A-8C2D-EA95CE753054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2802BC4-C2F1-434E-8945-136102CC395A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15150" yWindow="6230" windowWidth="18560" windowHeight="14150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -55,15 +68,9 @@
     <t>282x272x22mm</t>
   </si>
   <si>
-    <t>Bonus Special Op Pack [64225] (German)</t>
-  </si>
-  <si>
     <t>300x300x226mm</t>
   </si>
   <si>
-    <t>Earth Under Siege Core Box [72104] (English)</t>
-  </si>
-  <si>
     <t>Gametrayz Campaign Trays [72154]</t>
   </si>
   <si>
@@ -76,9 +83,6 @@
     <t>300x300x100mm</t>
   </si>
   <si>
-    <t>Nemesis Expansion [72105] (English)</t>
-  </si>
-  <si>
     <t>Plastic Token Pack [72562]</t>
   </si>
   <si>
@@ -109,22 +113,31 @@
     <t>170x130x31mm</t>
   </si>
   <si>
-    <t>Update Pack [72106] (English)</t>
-  </si>
-  <si>
     <t>300x300x125mm</t>
   </si>
   <si>
-    <t>World Killer Expansion [72100] (English)</t>
-  </si>
-  <si>
     <t>Weight (lbs)</t>
   </si>
   <si>
     <t>258x166x63mm</t>
   </si>
   <si>
-    <t>Operative Expansion Pack (English)</t>
+    <t xml:space="preserve">Bonus Special Op Pack [64225] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Earth Under Siege Core Box [72104] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operative Expansion Pack </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nemesis Expansion [72105] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update Pack [72106] </t>
+  </si>
+  <si>
+    <t xml:space="preserve">World Killer Expansion [72100] </t>
   </si>
 </sst>
 </file>
@@ -467,12 +480,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
-    <col min="2" max="2" width="43.6640625" customWidth="1"/>
-    <col min="3" max="3" width="23.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="70.109375" customWidth="1"/>
+    <col min="2" max="2" width="43.6328125" customWidth="1"/>
+    <col min="3" max="3" width="23.6328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="70.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -483,7 +496,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -532,7 +545,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
@@ -543,10 +556,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" s="1">
         <v>11.5</v>
@@ -554,10 +567,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C8" s="1">
         <v>1.7</v>
@@ -565,10 +578,10 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1">
         <v>1.8</v>
@@ -576,7 +589,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
@@ -587,10 +600,10 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C11" s="1">
         <v>2.98</v>
@@ -598,10 +611,10 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C12" s="1">
         <v>0.27</v>
@@ -609,10 +622,10 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C13" s="1">
         <v>0.27</v>
@@ -620,10 +633,10 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C14" s="1">
         <v>0.67</v>
@@ -631,10 +644,10 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C15" s="1">
         <v>0.88</v>
@@ -642,10 +655,10 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C16" s="1">
         <v>0.88</v>
@@ -653,10 +666,10 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C17" s="1">
         <v>0.22</v>
@@ -664,7 +677,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B18" t="s">
         <v>10</v>
@@ -675,10 +688,10 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C19" s="1">
         <v>4.92</v>

</xml_diff>